<commit_message>
Reset Excel Table for MILLING-02
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-02.xlsx
+++ b/FM-MN-07_MILLING-02.xlsx
@@ -1775,11 +1775,7 @@
           <t>Worm Spindle ก่อนเริมงาน ตรวจสอบความ ผิดปกติของชุด  Back gauge  และ Motor</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="24" t="inlineStr"/>
       <c r="D6" s="24" t="inlineStr"/>
       <c r="E6" s="24" t="inlineStr"/>
       <c r="F6" s="24" t="inlineStr"/>
@@ -1820,11 +1816,7 @@
           <t>เช็ค Auto  Up-Down back gauge  และ Manual ( ความคร่องตัวในการเคลื่อนที่ของ Spindle )</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="24" t="inlineStr"/>
       <c r="D7" s="24" t="inlineStr"/>
       <c r="E7" s="24" t="inlineStr"/>
       <c r="F7" s="24" t="inlineStr"/>
@@ -1865,11 +1857,7 @@
           <t>ตรวจสอบการ SLIDE  ของแกน X</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="24" t="inlineStr"/>
       <c r="D8" s="24" t="inlineStr"/>
       <c r="E8" s="24" t="inlineStr"/>
       <c r="F8" s="24" t="inlineStr"/>
@@ -1910,11 +1898,7 @@
           <t>ตรวจสอบการ SLIDE  ของแกน Y</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="24" t="inlineStr"/>
       <c r="D9" s="24" t="inlineStr"/>
       <c r="E9" s="24" t="inlineStr"/>
       <c r="F9" s="24" t="inlineStr"/>
@@ -1955,11 +1939,7 @@
           <t>ตรวจสอบการ SLIDE  ของแกน Z</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="24" t="inlineStr"/>
       <c r="D10" s="24" t="inlineStr"/>
       <c r="E10" s="24" t="inlineStr"/>
       <c r="F10" s="24" t="inlineStr"/>
@@ -2000,11 +1980,7 @@
           <t>ระดับน้ำมันไฮดรอลิค ตรวจสอบน้ำมันในปั้มน้ำมันหล่อ ลื่นแกน  X,Y,Z</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C11" s="24" t="inlineStr"/>
       <c r="D11" s="24" t="inlineStr"/>
       <c r="E11" s="24" t="inlineStr"/>
       <c r="F11" s="24" t="inlineStr"/>
@@ -2045,11 +2021,7 @@
           <t>ตรวจน้ำมันหล่อลื่นเย็น ตรวจสอบการทำงานของปั้ม COOLANT และสภาพของน้ำ  COOLANT</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="C12" s="24" t="inlineStr"/>
       <c r="D12" s="24" t="inlineStr"/>
       <c r="E12" s="24" t="inlineStr"/>
       <c r="F12" s="24" t="inlineStr"/>
@@ -2090,11 +2062,7 @@
           <t>ตรวจสอบหน้าจอ  DIGITAL READ OUT และการทำ งานของ LINEAR SCALE</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C13" s="26" t="inlineStr"/>
       <c r="D13" s="25" t="inlineStr"/>
       <c r="E13" s="25" t="inlineStr"/>
       <c r="F13" s="25" t="inlineStr"/>
@@ -2135,11 +2103,7 @@
           <t>หยอดน้ำมันหล่อลื่นทุกวันจันทร์</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C14" s="26" t="inlineStr"/>
       <c r="D14" s="25" t="inlineStr"/>
       <c r="E14" s="25" t="inlineStr"/>
       <c r="F14" s="25" t="inlineStr"/>
@@ -2180,11 +2144,7 @@
           <t>ตรวจสอบการทำงานของไฟฟ้าแสงสว่างของเครื่อง</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C15" s="26" t="inlineStr"/>
       <c r="D15" s="25" t="inlineStr"/>
       <c r="E15" s="25" t="inlineStr"/>
       <c r="F15" s="25" t="inlineStr"/>
@@ -2225,11 +2185,7 @@
           <t>ตรวจสอบสภาพความพร้อมโดยรวมของเครื่องจักร  และอุกรณ์เสริมต่าง ๆ</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C16" s="26" t="inlineStr"/>
       <c r="D16" s="25" t="inlineStr"/>
       <c r="E16" s="25" t="inlineStr"/>
       <c r="F16" s="25" t="inlineStr"/>
@@ -2264,11 +2220,7 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="13" t="n"/>
       <c r="B17" s="12" t="n"/>
-      <c r="C17" s="36" t="inlineStr">
-        <is>
-          <t>ขวัญชัย</t>
-        </is>
-      </c>
+      <c r="C17" s="36" t="inlineStr"/>
       <c r="D17" s="9" t="inlineStr"/>
       <c r="E17" s="9" t="inlineStr"/>
       <c r="F17" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for MILLING-02 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-02.xlsx
+++ b/FM-MN-07_MILLING-02.xlsx
@@ -1780,7 +1780,11 @@
       <c r="E6" s="24" t="inlineStr"/>
       <c r="F6" s="24" t="inlineStr"/>
       <c r="G6" s="24" t="inlineStr"/>
-      <c r="H6" s="24" t="inlineStr"/>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="24" t="inlineStr"/>
       <c r="J6" s="24" t="inlineStr"/>
       <c r="K6" s="24" t="inlineStr"/>
@@ -1821,7 +1825,11 @@
       <c r="E7" s="24" t="inlineStr"/>
       <c r="F7" s="24" t="inlineStr"/>
       <c r="G7" s="24" t="inlineStr"/>
-      <c r="H7" s="24" t="inlineStr"/>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="24" t="inlineStr"/>
       <c r="J7" s="24" t="inlineStr"/>
       <c r="K7" s="24" t="inlineStr"/>
@@ -1862,7 +1870,11 @@
       <c r="E8" s="24" t="inlineStr"/>
       <c r="F8" s="24" t="inlineStr"/>
       <c r="G8" s="24" t="inlineStr"/>
-      <c r="H8" s="24" t="inlineStr"/>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="24" t="inlineStr"/>
       <c r="J8" s="24" t="inlineStr"/>
       <c r="K8" s="24" t="inlineStr"/>
@@ -1903,7 +1915,11 @@
       <c r="E9" s="24" t="inlineStr"/>
       <c r="F9" s="24" t="inlineStr"/>
       <c r="G9" s="24" t="inlineStr"/>
-      <c r="H9" s="24" t="inlineStr"/>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="24" t="inlineStr"/>
       <c r="J9" s="24" t="inlineStr"/>
       <c r="K9" s="24" t="inlineStr"/>
@@ -1944,7 +1960,11 @@
       <c r="E10" s="24" t="inlineStr"/>
       <c r="F10" s="24" t="inlineStr"/>
       <c r="G10" s="24" t="inlineStr"/>
-      <c r="H10" s="24" t="inlineStr"/>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="24" t="inlineStr"/>
       <c r="J10" s="24" t="inlineStr"/>
       <c r="K10" s="24" t="inlineStr"/>
@@ -1985,7 +2005,11 @@
       <c r="E11" s="24" t="inlineStr"/>
       <c r="F11" s="24" t="inlineStr"/>
       <c r="G11" s="24" t="inlineStr"/>
-      <c r="H11" s="24" t="inlineStr"/>
+      <c r="H11" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="24" t="inlineStr"/>
       <c r="J11" s="24" t="inlineStr"/>
       <c r="K11" s="24" t="inlineStr"/>
@@ -2026,7 +2050,11 @@
       <c r="E12" s="24" t="inlineStr"/>
       <c r="F12" s="24" t="inlineStr"/>
       <c r="G12" s="24" t="inlineStr"/>
-      <c r="H12" s="24" t="inlineStr"/>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I12" s="24" t="inlineStr"/>
       <c r="J12" s="24" t="inlineStr"/>
       <c r="K12" s="24" t="inlineStr"/>
@@ -2067,7 +2095,11 @@
       <c r="E13" s="25" t="inlineStr"/>
       <c r="F13" s="25" t="inlineStr"/>
       <c r="G13" s="25" t="inlineStr"/>
-      <c r="H13" s="25" t="inlineStr"/>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="25" t="inlineStr"/>
       <c r="J13" s="25" t="inlineStr"/>
       <c r="K13" s="25" t="inlineStr"/>
@@ -2108,7 +2140,11 @@
       <c r="E14" s="25" t="inlineStr"/>
       <c r="F14" s="25" t="inlineStr"/>
       <c r="G14" s="25" t="inlineStr"/>
-      <c r="H14" s="25" t="inlineStr"/>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="25" t="inlineStr"/>
       <c r="J14" s="25" t="inlineStr"/>
       <c r="K14" s="25" t="inlineStr"/>
@@ -2149,7 +2185,11 @@
       <c r="E15" s="25" t="inlineStr"/>
       <c r="F15" s="25" t="inlineStr"/>
       <c r="G15" s="25" t="inlineStr"/>
-      <c r="H15" s="25" t="inlineStr"/>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="25" t="inlineStr"/>
       <c r="J15" s="25" t="inlineStr"/>
       <c r="K15" s="25" t="inlineStr"/>
@@ -2190,7 +2230,11 @@
       <c r="E16" s="25" t="inlineStr"/>
       <c r="F16" s="25" t="inlineStr"/>
       <c r="G16" s="25" t="inlineStr"/>
-      <c r="H16" s="25" t="inlineStr"/>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="25" t="inlineStr"/>
       <c r="J16" s="25" t="inlineStr"/>
       <c r="K16" s="25" t="inlineStr"/>
@@ -2225,7 +2269,11 @@
       <c r="E17" s="9" t="inlineStr"/>
       <c r="F17" s="9" t="inlineStr"/>
       <c r="G17" s="9" t="inlineStr"/>
-      <c r="H17" s="9" t="inlineStr"/>
+      <c r="H17" s="36" t="inlineStr">
+        <is>
+          <t>นาย ทินภัทร สียางนอก</t>
+        </is>
+      </c>
       <c r="I17" s="9" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-02 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-02.xlsx
+++ b/FM-MN-07_MILLING-02.xlsx
@@ -1785,7 +1785,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="24" t="inlineStr"/>
+      <c r="I6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="24" t="inlineStr"/>
       <c r="K6" s="24" t="inlineStr"/>
       <c r="L6" s="24" t="inlineStr"/>
@@ -1830,7 +1834,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="24" t="inlineStr"/>
+      <c r="I7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="24" t="inlineStr"/>
       <c r="K7" s="24" t="inlineStr"/>
       <c r="L7" s="24" t="inlineStr"/>
@@ -1875,7 +1883,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="24" t="inlineStr"/>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="24" t="inlineStr"/>
       <c r="K8" s="24" t="inlineStr"/>
       <c r="L8" s="24" t="inlineStr"/>
@@ -1920,7 +1932,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="24" t="inlineStr"/>
+      <c r="I9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="24" t="inlineStr"/>
       <c r="K9" s="24" t="inlineStr"/>
       <c r="L9" s="24" t="inlineStr"/>
@@ -1965,7 +1981,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="24" t="inlineStr"/>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="24" t="inlineStr"/>
       <c r="K10" s="24" t="inlineStr"/>
       <c r="L10" s="24" t="inlineStr"/>
@@ -2010,7 +2030,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="24" t="inlineStr"/>
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="24" t="inlineStr"/>
       <c r="K11" s="24" t="inlineStr"/>
       <c r="L11" s="24" t="inlineStr"/>
@@ -2055,7 +2079,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I12" s="24" t="inlineStr"/>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J12" s="24" t="inlineStr"/>
       <c r="K12" s="24" t="inlineStr"/>
       <c r="L12" s="24" t="inlineStr"/>
@@ -2100,7 +2128,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="25" t="inlineStr"/>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="25" t="inlineStr"/>
       <c r="K13" s="25" t="inlineStr"/>
       <c r="L13" s="25" t="inlineStr"/>
@@ -2145,7 +2177,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I14" s="25" t="inlineStr"/>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J14" s="25" t="inlineStr"/>
       <c r="K14" s="25" t="inlineStr"/>
       <c r="L14" s="25" t="inlineStr"/>
@@ -2190,7 +2226,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I15" s="25" t="inlineStr"/>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J15" s="25" t="inlineStr"/>
       <c r="K15" s="25" t="inlineStr"/>
       <c r="L15" s="25" t="inlineStr"/>
@@ -2235,7 +2275,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I16" s="25" t="inlineStr"/>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J16" s="25" t="inlineStr"/>
       <c r="K16" s="25" t="inlineStr"/>
       <c r="L16" s="25" t="inlineStr"/>
@@ -2274,7 +2318,11 @@
           <t>นาย ทินภัทร สียางนอก</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr"/>
+      <c r="I17" s="36" t="inlineStr">
+        <is>
+          <t>นาย ทินภัทร สียางนอก</t>
+        </is>
+      </c>
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr"/>
       <c r="L17" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-02 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-02.xlsx
+++ b/FM-MN-07_MILLING-02.xlsx
@@ -1790,7 +1790,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="24" t="inlineStr"/>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="24" t="inlineStr"/>
       <c r="L6" s="24" t="inlineStr"/>
       <c r="M6" s="24" t="inlineStr"/>
@@ -1839,7 +1843,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="24" t="inlineStr"/>
+      <c r="J7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="24" t="inlineStr"/>
       <c r="L7" s="24" t="inlineStr"/>
       <c r="M7" s="24" t="inlineStr"/>
@@ -1888,7 +1896,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="24" t="inlineStr"/>
+      <c r="J8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="24" t="inlineStr"/>
       <c r="L8" s="24" t="inlineStr"/>
       <c r="M8" s="24" t="inlineStr"/>
@@ -1937,7 +1949,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="24" t="inlineStr"/>
+      <c r="J9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="24" t="inlineStr"/>
       <c r="L9" s="24" t="inlineStr"/>
       <c r="M9" s="24" t="inlineStr"/>
@@ -1986,7 +2002,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="24" t="inlineStr"/>
+      <c r="J10" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="24" t="inlineStr"/>
       <c r="L10" s="24" t="inlineStr"/>
       <c r="M10" s="24" t="inlineStr"/>
@@ -2035,7 +2055,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="24" t="inlineStr"/>
+      <c r="J11" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="24" t="inlineStr"/>
       <c r="L11" s="24" t="inlineStr"/>
       <c r="M11" s="24" t="inlineStr"/>
@@ -2084,7 +2108,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J12" s="24" t="inlineStr"/>
+      <c r="J12" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K12" s="24" t="inlineStr"/>
       <c r="L12" s="24" t="inlineStr"/>
       <c r="M12" s="24" t="inlineStr"/>
@@ -2133,7 +2161,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="25" t="inlineStr"/>
+      <c r="J13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="25" t="inlineStr"/>
       <c r="L13" s="25" t="inlineStr"/>
       <c r="M13" s="25" t="inlineStr"/>
@@ -2182,7 +2214,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J14" s="25" t="inlineStr"/>
+      <c r="J14" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="25" t="inlineStr"/>
       <c r="L14" s="25" t="inlineStr"/>
       <c r="M14" s="25" t="inlineStr"/>
@@ -2231,7 +2267,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J15" s="25" t="inlineStr"/>
+      <c r="J15" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="25" t="inlineStr"/>
       <c r="L15" s="25" t="inlineStr"/>
       <c r="M15" s="25" t="inlineStr"/>
@@ -2280,7 +2320,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J16" s="25" t="inlineStr"/>
+      <c r="J16" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="25" t="inlineStr"/>
       <c r="L16" s="25" t="inlineStr"/>
       <c r="M16" s="25" t="inlineStr"/>
@@ -2428,7 +2472,11 @@
       <c r="G20" s="32" t="n"/>
       <c r="H20" s="32" t="n"/>
       <c r="I20" s="32" t="n"/>
-      <c r="J20" s="32" t="n"/>
+      <c r="J20" s="36" t="inlineStr">
+        <is>
+          <t>นาย ทินภัทร สียางนอก</t>
+        </is>
+      </c>
       <c r="K20" s="32" t="n"/>
       <c r="L20" s="32" t="n"/>
       <c r="M20" s="32" t="n"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-02 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-02.xlsx
+++ b/FM-MN-07_MILLING-02.xlsx
@@ -355,7 +355,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -463,6 +463,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1796,7 +1799,11 @@
         </is>
       </c>
       <c r="K6" s="24" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="24" t="inlineStr"/>
       <c r="N6" s="24" t="inlineStr"/>
       <c r="O6" s="24" t="inlineStr"/>
@@ -1849,7 +1856,11 @@
         </is>
       </c>
       <c r="K7" s="24" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr"/>
+      <c r="L7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="24" t="inlineStr"/>
       <c r="N7" s="24" t="inlineStr"/>
       <c r="O7" s="24" t="inlineStr"/>
@@ -1902,7 +1913,11 @@
         </is>
       </c>
       <c r="K8" s="24" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="24" t="inlineStr"/>
       <c r="N8" s="24" t="inlineStr"/>
       <c r="O8" s="24" t="inlineStr"/>
@@ -1955,7 +1970,11 @@
         </is>
       </c>
       <c r="K9" s="24" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr"/>
+      <c r="L9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="24" t="inlineStr"/>
       <c r="N9" s="24" t="inlineStr"/>
       <c r="O9" s="24" t="inlineStr"/>
@@ -2008,7 +2027,11 @@
         </is>
       </c>
       <c r="K10" s="24" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr"/>
+      <c r="L10" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="24" t="inlineStr"/>
       <c r="N10" s="24" t="inlineStr"/>
       <c r="O10" s="24" t="inlineStr"/>
@@ -2061,7 +2084,11 @@
         </is>
       </c>
       <c r="K11" s="24" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr"/>
+      <c r="L11" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M11" s="24" t="inlineStr"/>
       <c r="N11" s="24" t="inlineStr"/>
       <c r="O11" s="24" t="inlineStr"/>
@@ -2114,7 +2141,11 @@
         </is>
       </c>
       <c r="K12" s="24" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr"/>
+      <c r="L12" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M12" s="24" t="inlineStr"/>
       <c r="N12" s="24" t="inlineStr"/>
       <c r="O12" s="24" t="inlineStr"/>
@@ -2167,7 +2198,11 @@
         </is>
       </c>
       <c r="K13" s="25" t="inlineStr"/>
-      <c r="L13" s="25" t="inlineStr"/>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="25" t="inlineStr"/>
       <c r="N13" s="25" t="inlineStr"/>
       <c r="O13" s="25" t="inlineStr"/>
@@ -2220,7 +2255,11 @@
         </is>
       </c>
       <c r="K14" s="25" t="inlineStr"/>
-      <c r="L14" s="25" t="inlineStr"/>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="25" t="inlineStr"/>
       <c r="N14" s="25" t="inlineStr"/>
       <c r="O14" s="25" t="inlineStr"/>
@@ -2273,7 +2312,11 @@
         </is>
       </c>
       <c r="K15" s="25" t="inlineStr"/>
-      <c r="L15" s="25" t="inlineStr"/>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="25" t="inlineStr"/>
       <c r="N15" s="25" t="inlineStr"/>
       <c r="O15" s="25" t="inlineStr"/>
@@ -2326,7 +2369,11 @@
         </is>
       </c>
       <c r="K16" s="25" t="inlineStr"/>
-      <c r="L16" s="25" t="inlineStr"/>
+      <c r="L16" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="25" t="inlineStr"/>
       <c r="N16" s="25" t="inlineStr"/>
       <c r="O16" s="25" t="inlineStr"/>
@@ -2478,7 +2525,11 @@
         </is>
       </c>
       <c r="K20" s="32" t="n"/>
-      <c r="L20" s="32" t="n"/>
+      <c r="L20" s="36" t="inlineStr">
+        <is>
+          <t>นาย ทินภัทร สียางนอก</t>
+        </is>
+      </c>
       <c r="M20" s="32" t="n"/>
       <c r="N20" s="32" t="n"/>
       <c r="O20" s="32" t="n"/>
@@ -2611,7 +2662,11 @@
       </c>
     </row>
     <row r="25" ht="240.75" customHeight="1">
-      <c r="B25" s="43" t="n"/>
+      <c r="B25" s="45" t="inlineStr">
+        <is>
+          <t>[วันที่ 10]: ข้อ 6: ขาโช๊คปั้มน้ำมันเสียรอซ่อม</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.25" customHeight="1"/>
     <row r="27" ht="21" customHeight="1">

</xml_diff>